<commit_message>
feat: 更新购买记录 2026-07-18 03:15
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1269,7 +1269,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>截图</t>
+          <t>备注</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>3311879379799327755</t>
         </is>
       </c>
-      <c r="I3" s="7" t="n"/>
+      <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1347,7 +1347,7 @@
           <t>6928046994516508348</t>
         </is>
       </c>
-      <c r="I4" s="7" t="n"/>
+      <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1381,8 +1381,7 @@
           <t>2 笔订单</t>
         </is>
       </c>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="n"/>
@@ -7354,7 +7353,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H6:I6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 03:31
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -11,6 +11,7 @@
     <sheet name="📊月度统计" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="📈年度统计" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="🏪平台分布" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="📦出货记录" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -154,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -207,6 +210,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1264,12 +1270,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>订单号</t>
+          <t>购买订单号</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>关联出货单</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1381,7 +1387,8 @@
           <t>2 笔订单</t>
         </is>
       </c>
-      <c r="I6" s="14" t="n"/>
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="14" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="n"/>
@@ -7353,7 +7360,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H6:J6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8004,4 +8011,731 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N502"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>📦 出货记录表 (2026年)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>出货平台</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>订购日期</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>发货日期</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>商品名称</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>规格</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>销售价</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>税金</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>手续费</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>销售额</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>出货订单号</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>关联购买记录</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>500ml啤酒杯耐热耐冷足球奖杯杯</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>透明</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>6E-4EHX-JF04</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>184</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>312</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>1714</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>503-95444475-5097463</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>3311879379799327755</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n">
+        <v>46221</v>
+      </c>
+      <c r="D4" s="20" t="n">
+        <v>46224</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>500ml啤酒杯耐热耐冷足球奖杯杯</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>琥珀色</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>LK-RN2M-G3YX</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>184</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>312</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>1714</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>249-6387958-2579060</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>6928046994516508348</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>📊 合计</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>总销售额: ¥3,428.00</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>2 笔出货</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="A6:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 03:36
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -157,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -212,7 +211,10 @@
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1317,7 +1319,11 @@
           <t>3311879379799327755</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>503-95444475-5097463</t>
+        </is>
+      </c>
       <c r="J3" s="4" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1353,7 +1359,11 @@
           <t>6928046994516508348</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>249-6387958-2579060</t>
+        </is>
+      </c>
       <c r="J4" s="4" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -8110,10 +8120,10 @@
           <t>Amazon日本站</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="21" t="n">
         <v>46214</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="21" t="n">
         <v>46217</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -8166,10 +8176,10 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>46221</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="21" t="n">
         <v>46224</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -8228,11 +8238,15 @@
           <t>总销售额: ¥3,428.00</t>
         </is>
       </c>
+      <c r="J6" s="13" t="n"/>
+      <c r="K6" s="13" t="n"/>
+      <c r="L6" s="14" t="n"/>
       <c r="M6" s="10" t="inlineStr">
         <is>
           <t>2 笔出货</t>
         </is>
       </c>
+      <c r="N6" s="14" t="n"/>
     </row>
     <row r="7"/>
     <row r="8"/>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 03:37
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1319,7 +1319,7 @@
           <t>3311879379799327755</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>503-95444475-5097463</t>
         </is>
@@ -1359,7 +1359,7 @@
           <t>6928046994516508348</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>249-6387958-2579060</t>
         </is>
@@ -7372,6 +7372,10 @@
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:J6"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8161,7 +8165,7 @@
           <t>503-95444475-5097463</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>3311879379799327755</t>
         </is>
@@ -8217,7 +8221,7 @@
           <t>249-6387958-2579060</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>6928046994516508348</t>
         </is>
@@ -8750,6 +8754,10 @@
     <mergeCell ref="I6:L6"/>
     <mergeCell ref="A6:D6"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 03:48
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1215,22 +1215,22 @@
   <dimension ref="A1:J504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🛒 购买记录明细表  (2026年)</t>
+          <t>🛒 购买记录明细表 (2026年)</t>
         </is>
       </c>
     </row>
@@ -7368,13 +7368,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="H6:J6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId2"/>
+    <hyperlink ref="I3" location="'📦出货记录'!A3" display="503-95444475-5097463"/>
+    <hyperlink ref="I4" location="'📦出货记录'!A4" display="249-6387958-2579060"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7388,6 +7389,22 @@
   </sheetPr>
   <dimension ref="A1:N502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
@@ -8102,14 +8119,15 @@
     <row r="501"/>
     <row r="502"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="I6:L6"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="I6:L6"/>
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
+    <hyperlink ref="N3" location="'🛒购买记录明细'!A3" display="3311879379799327755"/>
+    <hyperlink ref="N4" location="'🛒购买记录明细'!A4" display="6928046994516508348"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 04:00
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="&quot;JPY&quot; #,##0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -156,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -215,6 +216,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7398,10 +7402,10 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
@@ -7456,22 +7460,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>销售价</t>
+          <t>销售价(日元)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>税金</t>
+          <t>税金(日元)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>手续费</t>
+          <t>手续费(日元)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>销售额</t>
+          <t>销售额(日元)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -7518,16 +7522,16 @@
       <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="22" t="n">
         <v>2026</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="22" t="n">
         <v>184</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="K3" s="22" t="n">
         <v>312</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="L3" s="22" t="n">
         <v>1714</v>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -7574,16 +7578,16 @@
       <c r="H4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="22" t="n">
         <v>2026</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="22" t="n">
         <v>184</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="K4" s="22" t="n">
         <v>312</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="L4" s="22" t="n">
         <v>1714</v>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -7609,7 +7613,7 @@
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>总销售额: ¥3,428.00</t>
+          <t>总销售额: JPY 3,428</t>
         </is>
       </c>
       <c r="J6" s="13" t="n"/>
@@ -8120,9 +8124,9 @@
     <row r="502"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="I6:L6"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="M6:N6"/>
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 06:15
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,11 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="&quot;JPY&quot; #,##0"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1222,11 +1223,11 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
@@ -1371,50 +1372,71 @@
       <c r="J4" s="4" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="7" t="n"/>
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>拼多多</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>46221.59108796297</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>260718-641864876461684</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>249-6387958-2579060</t>
+        </is>
+      </c>
       <c r="J5" s="4" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="10" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="9" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>2 笔订单</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="14" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="9" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>3 笔订单</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="14" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="3" t="n"/>
@@ -7373,13 +7395,14 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I3" location="'📦出货记录'!A3" display="503-95444475-5097463"/>
     <hyperlink ref="I4" location="'📦出货记录'!A4" display="249-6387958-2579060"/>
+    <hyperlink ref="I5" location="'📦出货记录'!A4" display="249-6387958-2579060"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8335,13 +8358,13 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>17.4</v>
+        <v>37.4</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>8.699999999999999</v>
+        <v>12.47</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>1</v>
@@ -8465,13 +8488,13 @@
       </c>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>17.4</v>
+        <v>37.4</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>8.699999999999999</v>
+        <v>12.47</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>1</v>
@@ -8545,13 +8568,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>17.4</v>
+        <v>37.4</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>8.699999999999999</v>
+        <v>12.47</v>
       </c>
       <c r="E3" s="3" t="n"/>
     </row>
@@ -8640,7 +8663,7 @@
         <v>11.5</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>0.6609</v>
+        <v>0.3075</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -8656,7 +8679,7 @@
         <v>5.9</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>0.3391</v>
+        <v>0.1578</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -8698,13 +8721,13 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0</v>
+        <v>0.5348000000000001</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -8762,10 +8785,10 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>17.4</v>
+        <v>37.4</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-18 06:17
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,12 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="&quot;JPY&quot; #,##0"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1221,7 +1220,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
@@ -1337,31 +1336,31 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>抖音商城</t>
+          <t>拼多多</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>46221.42550925926</v>
+        <v>46221.59108796297</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>创意大力神杯世界杯足球杯</t>
+          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>500ml琥珀圆形大力神杯(牛皮纸盒包装)</t>
+          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>11.5</v>
+        <v>20</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>6928046994516508348</t>
+          <t>260718-641864876461684</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -1372,71 +1371,43 @@
       <c r="J4" s="4" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>拼多多</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="n">
-        <v>46221.59108796297</v>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>260718-641864876461684</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>249-6387958-2579060</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="7" t="n"/>
       <c r="J5" s="4" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="10" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>📊 合计</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="9" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>2 笔订单</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="14" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>📊 合计</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="n"/>
-      <c r="C7" s="13" t="n"/>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="9" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>3 笔订单</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="14" t="n"/>
+      <c r="A7" s="10" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="3" t="n"/>
@@ -7395,9 +7366,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H6:J6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I3" location="'📦出货记录'!A3" display="503-95444475-5097463"/>
@@ -7430,7 +7401,7 @@
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -7620,7 +7591,7 @@
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>6928046994516508348</t>
+          <t>260718-641864876461684</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8125,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N3" location="'🛒购买记录明细'!A3" display="3311879379799327755"/>
-    <hyperlink ref="N4" location="'🛒购买记录明细'!A4" display="6928046994516508348"/>
+    <hyperlink ref="N4" location="'🛒购买记录明细'!A4" display="260718-641864876461684"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8358,13 +8329,13 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>37.4</v>
+        <v>25.9</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>12.47</v>
+        <v>12.95</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>1</v>
@@ -8488,13 +8459,13 @@
       </c>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>37.4</v>
+        <v>25.9</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>12.47</v>
+        <v>12.95</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>1</v>
@@ -8568,13 +8539,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>37.4</v>
+        <v>25.9</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>12.47</v>
+        <v>12.95</v>
       </c>
       <c r="E3" s="3" t="n"/>
     </row>
@@ -8657,13 +8628,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>11.5</v>
+        <v>0</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>0.3075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -8679,7 +8650,7 @@
         <v>5.9</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>0.1578</v>
+        <v>0.2278</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -8727,7 +8698,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.5348000000000001</v>
+        <v>0.7722</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -8785,10 +8756,10 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>37.4</v>
+        <v>25.9</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-21 03:09
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,11 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="&quot;JPY&quot; #,##0"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1216,7 +1217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J504"/>
+  <dimension ref="A1:L504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1229,6 +1230,8 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1266,7 +1269,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>购买数量</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1285,6 +1288,16 @@
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>出货数量</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>库存</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1328,7 +1341,13 @@
           <t>503-95444475-5097463</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1368,46 +1387,98 @@
           <t>249-6387958-2579060</t>
         </is>
       </c>
-      <c r="J4" s="4" t="n"/>
+      <c r="J4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1688</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>46224.4587962963</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>玻璃修复膏玻璃表面专业抛光</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>50g+海绵</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>3313191614834136171</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>249-4866874-7926210</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>最低起订2个，卖出1个，库存1个</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="10" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="9" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>2 笔订单</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="14" t="n"/>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="10" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="9" t="n">
+        <v>37.79</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>3 笔订单</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>库存合计</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="3" t="n"/>
@@ -7366,14 +7437,14 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I3" location="'📦出货记录'!A3" display="503-95444475-5097463"/>
     <hyperlink ref="I4" location="'📦出货记录'!A4" display="249-6387958-2579060"/>
-    <hyperlink ref="I5" location="'📦出货记录'!A4" display="249-6387958-2579060"/>
+    <hyperlink ref="I5" location="'📦出货记录'!A5" display="249-4866874-7926210"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7595,32 +7666,88 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>46223</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>46225</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>玻璃修复膏 50g 车用</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>50g</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>1X-GB0W-BY30</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>1122</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>102</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>117</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>1005</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>249-4866874-7926210</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>3313191614834136171</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="8" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="M6" s="10" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="H6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 3,428</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="n"/>
-      <c r="K6" s="13" t="n"/>
-      <c r="L6" s="14" t="n"/>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>2 笔出货</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="n"/>
-    </row>
-    <row r="7"/>
+      <c r="H7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 4,433</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>3 笔出货</t>
+        </is>
+      </c>
+    </row>
     <row r="8"/>
     <row r="9"/>
     <row r="10"/>
@@ -8118,14 +8245,15 @@
     <row r="502"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="I7:L7"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A6:D6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N3" location="'🛒购买记录明细'!A3" display="3311879379799327755"/>
     <hyperlink ref="N4" location="'🛒购买记录明细'!A4" display="260718-641864876461684"/>
+    <hyperlink ref="N5" location="'🛒购买记录明细'!A5" display="3313191614834136171"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8329,13 +8457,13 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>25.9</v>
+        <v>37.79</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>12.95</v>
+        <v>12.6</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>1</v>
@@ -8459,13 +8587,13 @@
       </c>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>25.9</v>
+        <v>37.79</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>12.95</v>
+        <v>12.6</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>1</v>
@@ -8539,13 +8667,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>25.9</v>
+        <v>37.79</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>12.95</v>
+        <v>12.6</v>
       </c>
       <c r="E3" s="3" t="n"/>
     </row>
@@ -8644,13 +8772,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>5.9</v>
+        <v>17.79</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>0.2278</v>
+        <v>0.4708</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -8698,7 +8826,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.7722</v>
+        <v>0.5292</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -8756,10 +8884,10 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>25.9</v>
+        <v>37.79</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat: 更新购买记录 2026-07-21 03:14
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -20,12 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="&quot;JPY&quot; #,##0"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1342,7 +1341,7 @@
         </is>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>0</v>
@@ -1388,7 +1387,7 @@
         </is>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>0</v>
@@ -7438,8 +7437,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I3" location="'📦出货记录'!A3" display="503-95444475-5097463"/>
@@ -7742,11 +7741,15 @@
           <t>总销售额: JPY 4,433</t>
         </is>
       </c>
+      <c r="J7" s="13" t="n"/>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="14" t="n"/>
       <c r="M7" s="10" t="inlineStr">
         <is>
           <t>3 笔出货</t>
         </is>
       </c>
+      <c r="N7" s="14" t="n"/>
     </row>
     <row r="8"/>
     <row r="9"/>
@@ -8245,8 +8248,8 @@
     <row r="502"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="M7:N7"/>
     <mergeCell ref="I7:L7"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: 新增出货订单 249-3982035-2006207 切蒜器
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1968,25 +1968,76 @@
       </c>
       <c r="N14" s="27" t="n"/>
     </row>
-    <row r="15"/>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>46241</v>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G15" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J15" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K15" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L15" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>249-3982035-2006207</t>
+        </is>
+      </c>
+      <c r="N15" s="27" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I16" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 12,870</t>
-        </is>
-      </c>
-      <c r="M16" s="32" t="inlineStr">
-        <is>
-          <t>12 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 13,799</t>
+        </is>
+      </c>
+      <c r="M17" s="32" t="inlineStr">
+        <is>
+          <t>13 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
@@ -2174,9 +2225,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="I16:L16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="I17:L17"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2266,7 +2317,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.46</v>
@@ -2275,11 +2326,11 @@
         <v>46236.88541666666</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46236</v>
+        <v>46239</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (8个)</t>
+          <t>库存充足 (7个)</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2438,7 @@
         </is>
       </c>
       <c r="D8" s="32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="32" t="inlineStr">
         <is>
@@ -3075,21 +3126,54 @@
         <v>929</v>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>3315760069697054152</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>249-3982035-2006207</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="29" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H15" s="34" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G16" s="31" t="n">
-        <v>72.64</v>
-      </c>
-      <c r="H16" s="35" t="n">
-        <v>12870</v>
-      </c>
-    </row>
-    <row r="17"/>
+      <c r="G17" s="31" t="n">
+        <v>77.20999999999999</v>
+      </c>
+      <c r="H17" s="35" t="n">
+        <v>13799</v>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
@@ -3277,7 +3361,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3305,6 +3389,8 @@
     <hyperlink ref="C13" location="'📤销售表'!A13" display="503-5593381-1019045"/>
     <hyperlink ref="B14" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C14" location="'📤销售表'!A14" display="249-4191194-8245444"/>
+    <hyperlink ref="B15" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C15" location="'📤销售表'!A15" display="249-3982035-2006207"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增出货订单 250-0207357-6815003 切蒜器
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2020,25 +2020,76 @@
       </c>
       <c r="N15" s="27" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G16" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J16" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K16" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L16" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>250-0207357-6815003</t>
+        </is>
+      </c>
+      <c r="N16" s="27" t="n"/>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I17" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 13,799</t>
-        </is>
-      </c>
-      <c r="M17" s="32" t="inlineStr">
-        <is>
-          <t>13 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="I18" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 14,728</t>
+        </is>
+      </c>
+      <c r="M18" s="32" t="inlineStr">
+        <is>
+          <t>14 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="19"/>
     <row r="20"/>
     <row r="21"/>
@@ -2225,9 +2276,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="I18:L18"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2317,7 +2368,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.46</v>
@@ -2326,11 +2377,11 @@
         <v>46236.88541666666</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (7个)</t>
+          <t>库存充足 (6个)</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2489,7 @@
         </is>
       </c>
       <c r="D8" s="32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="32" t="inlineStr">
         <is>
@@ -3160,21 +3211,54 @@
         <v>929</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>3315760069697054152</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr">
+        <is>
+          <t>250-0207357-6815003</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="29" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H16" s="34" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G17" s="31" t="n">
-        <v>77.20999999999999</v>
-      </c>
-      <c r="H17" s="35" t="n">
-        <v>13799</v>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="G18" s="31" t="n">
+        <v>81.78</v>
+      </c>
+      <c r="H18" s="35" t="n">
+        <v>14728</v>
+      </c>
+    </row>
     <row r="19"/>
     <row r="20"/>
     <row r="21"/>
@@ -3361,7 +3445,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3391,6 +3475,8 @@
     <hyperlink ref="C14" location="'📤销售表'!A14" display="249-4191194-8245444"/>
     <hyperlink ref="B15" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C15" location="'📤销售表'!A15" display="249-3982035-2006207"/>
+    <hyperlink ref="B16" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C16" location="'📤销售表'!A16" display="250-0207357-6815003"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增出货订单 250-6902845-9205438 切蒜器
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2072,25 +2072,76 @@
       </c>
       <c r="N16" s="27" t="n"/>
     </row>
-    <row r="17"/>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>46241</v>
+      </c>
+      <c r="D17" s="33" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J17" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K17" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L17" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>250-6902845-9205438</t>
+        </is>
+      </c>
+      <c r="N17" s="27" t="n"/>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I18" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 14,728</t>
-        </is>
-      </c>
-      <c r="M18" s="32" t="inlineStr">
-        <is>
-          <t>14 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+      <c r="I19" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 15,657</t>
+        </is>
+      </c>
+      <c r="M19" s="32" t="inlineStr">
+        <is>
+          <t>15 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="20"/>
     <row r="21"/>
     <row r="22"/>
@@ -2276,9 +2327,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="I18:L18"/>
+    <mergeCell ref="I19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2368,7 +2419,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.46</v>
@@ -2377,11 +2428,11 @@
         <v>46236.88541666666</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (6个)</t>
+          <t>库存充足 (5个)</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2540,7 @@
         </is>
       </c>
       <c r="D8" s="32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="32" t="inlineStr">
         <is>
@@ -3245,21 +3296,54 @@
         <v>929</v>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>3315760069697054152</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>250-6902845-9205438</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="29" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H17" s="34" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G18" s="31" t="n">
-        <v>81.78</v>
-      </c>
-      <c r="H18" s="35" t="n">
-        <v>14728</v>
-      </c>
-    </row>
-    <row r="19"/>
+      <c r="G19" s="31" t="n">
+        <v>86.34999999999999</v>
+      </c>
+      <c r="H19" s="35" t="n">
+        <v>15657</v>
+      </c>
+    </row>
     <row r="20"/>
     <row r="21"/>
     <row r="22"/>
@@ -3445,7 +3529,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3477,6 +3561,8 @@
     <hyperlink ref="C15" location="'📤销售表'!A15" display="249-3982035-2006207"/>
     <hyperlink ref="B16" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C16" location="'📤销售表'!A16" display="250-0207357-6815003"/>
+    <hyperlink ref="B17" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C17" location="'📤销售表'!A17" display="250-6902845-9205438"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增出货订单 250-3154848-2935021 切蒜器
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2124,25 +2124,76 @@
       </c>
       <c r="N17" s="27" t="n"/>
     </row>
-    <row r="18"/>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D18" s="33" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G18" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J18" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K18" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L18" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M18" s="25" t="inlineStr">
+        <is>
+          <t>250-3154848-2935021</t>
+        </is>
+      </c>
+      <c r="N18" s="27" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I19" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 15,657</t>
-        </is>
-      </c>
-      <c r="M19" s="32" t="inlineStr">
-        <is>
-          <t>15 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+      <c r="I20" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 16,586</t>
+        </is>
+      </c>
+      <c r="M20" s="32" t="inlineStr">
+        <is>
+          <t>16 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="21"/>
     <row r="22"/>
     <row r="23"/>
@@ -2327,9 +2378,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="I19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="I20:L20"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2419,7 +2470,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.46</v>
@@ -2428,11 +2479,11 @@
         <v>46236.88541666666</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46241</v>
+        <v>46243</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (5个)</t>
+          <t>库存充足 (4个)</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2591,7 @@
         </is>
       </c>
       <c r="D8" s="32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" s="32" t="inlineStr">
         <is>
@@ -3330,21 +3381,54 @@
         <v>929</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>3315760069697054152</t>
+        </is>
+      </c>
+      <c r="C18" s="36" t="inlineStr">
+        <is>
+          <t>250-3154848-2935021</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="29" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H18" s="34" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G19" s="31" t="n">
-        <v>86.34999999999999</v>
-      </c>
-      <c r="H19" s="35" t="n">
-        <v>15657</v>
-      </c>
-    </row>
-    <row r="20"/>
+      <c r="G20" s="31" t="n">
+        <v>90.92</v>
+      </c>
+      <c r="H20" s="35" t="n">
+        <v>16586</v>
+      </c>
+    </row>
     <row r="21"/>
     <row r="22"/>
     <row r="23"/>
@@ -3529,7 +3613,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3563,6 +3647,8 @@
     <hyperlink ref="C16" location="'📤销售表'!A16" display="250-0207357-6815003"/>
     <hyperlink ref="B17" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C17" location="'📤销售表'!A17" display="250-6902845-9205438"/>
+    <hyperlink ref="B18" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C18" location="'📤销售表'!A18" display="250-3154848-2935021"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增除黄剂采购3316792152573008960 & 销售249-8279106-7397442
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1022,23 +1022,60 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>1688</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>46244.33587962963</v>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>KineShineX塑料除黄剂</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>100ml+毛巾</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="H9" s="27" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="J9" s="27" t="n"/>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G10" s="31" t="n">
-        <v>115.2</v>
-      </c>
-      <c r="H10" s="32" t="inlineStr">
-        <is>
-          <t>6 笔进货</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+      <c r="G11" s="31" t="n">
+        <v>135.2</v>
+      </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>7 笔进货</t>
+        </is>
+      </c>
+    </row>
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
@@ -1232,9 +1269,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2176,25 +2213,76 @@
       </c>
       <c r="N18" s="27" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D19" s="33" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="G19" s="25" t="inlineStr">
+        <is>
+          <t>asd159</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="34" t="n">
+        <v>1468</v>
+      </c>
+      <c r="J19" s="34" t="n">
+        <v>134</v>
+      </c>
+      <c r="K19" s="34" t="n">
+        <v>194</v>
+      </c>
+      <c r="L19" s="34" t="n">
+        <v>1673</v>
+      </c>
+      <c r="M19" s="25" t="inlineStr">
+        <is>
+          <t>249-8279106-7397442</t>
+        </is>
+      </c>
+      <c r="N19" s="27" t="n"/>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I20" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 16,586</t>
-        </is>
-      </c>
-      <c r="M20" s="32" t="inlineStr">
-        <is>
-          <t>16 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="I21" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 18,259</t>
+        </is>
+      </c>
+      <c r="M21" s="32" t="inlineStr">
+        <is>
+          <t>17 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="22"/>
     <row r="23"/>
     <row r="24"/>
@@ -2378,9 +2466,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="I20:L20"/>
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="I21:L21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2493,29 +2581,29 @@
       </c>
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>KineShineX玻璃修复膏</t>
+          <t>KineShineX塑料除黄剂</t>
         </is>
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>50g+海绵</t>
+          <t>100ml+毛巾</t>
         </is>
       </c>
       <c r="D4" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="F4" s="33" t="n">
-        <v>46230.48587962963</v>
+        <v>46244.33587962963</v>
       </c>
       <c r="G4" s="33" t="n">
-        <v>46232</v>
+        <v>46242</v>
       </c>
       <c r="H4" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (1个)</t>
+          <t>库存充足 (2个)</t>
         </is>
       </c>
     </row>
@@ -2525,29 +2613,29 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>创意世界杯足球大力神杯</t>
+          <t>KineShineX玻璃修复膏</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>500ml透明圆形足球杯(牛皮纸盒包装)</t>
+          <t>50g+海绵</t>
         </is>
       </c>
       <c r="D5" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>46215.5080787037</v>
+        <v>46230.48587962963</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>46214</v>
+        <v>46232</v>
       </c>
       <c r="H5" s="27" t="inlineStr">
         <is>
-          <t>已售罄</t>
+          <t>库存充足 (1个)</t>
         </is>
       </c>
     </row>
@@ -2557,49 +2645,80 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
+          <t>创意世界杯足球大力神杯</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
+          <t>500ml透明圆形足球杯(牛皮纸盒包装)</t>
         </is>
       </c>
       <c r="D6" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="29" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>46215.5080787037</v>
+      </c>
+      <c r="G6" s="33" t="n">
+        <v>46214</v>
+      </c>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>已售罄</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F7" s="33" t="n">
         <v>46221.59108796297</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G7" s="33" t="n">
         <v>46221</v>
       </c>
-      <c r="H6" s="27" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
         <is>
           <t>已售罄</t>
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+    <row r="8"/>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>📊 库存合计</t>
         </is>
       </c>
-      <c r="D8" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="32" t="inlineStr">
-        <is>
-          <t>4 种商品</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+      <c r="D9" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>5 种商品</t>
+        </is>
+      </c>
+    </row>
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
@@ -2795,8 +2914,8 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="E9:H9"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3415,21 +3534,54 @@
         <v>929</v>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>249-8279106-7397442</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H19" s="34" t="n">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G20" s="31" t="n">
-        <v>90.92</v>
-      </c>
-      <c r="H20" s="35" t="n">
-        <v>16586</v>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="G21" s="31" t="n">
+        <v>97.59</v>
+      </c>
+      <c r="H21" s="35" t="n">
+        <v>18259</v>
+      </c>
+    </row>
     <row r="22"/>
     <row r="23"/>
     <row r="24"/>
@@ -3613,7 +3765,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3649,6 +3801,8 @@
     <hyperlink ref="C17" location="'📤销售表'!A17" display="250-6902845-9205438"/>
     <hyperlink ref="B18" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C18" location="'📤销售表'!A18" display="250-3154848-2935021"/>
+    <hyperlink ref="B19" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C19" location="'📤销售表'!A19" display="249-8279106-7397442"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增出货订单 503-5134375-2874203 塑料除黄剂
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2265,25 +2265,76 @@
       </c>
       <c r="N19" s="27" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="30" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D20" s="33" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="G20" s="25" t="inlineStr">
+        <is>
+          <t>asd159</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="34" t="n">
+        <v>1468</v>
+      </c>
+      <c r="J20" s="34" t="n">
+        <v>134</v>
+      </c>
+      <c r="K20" s="34" t="n">
+        <v>194</v>
+      </c>
+      <c r="L20" s="34" t="n">
+        <v>1673</v>
+      </c>
+      <c r="M20" s="25" t="inlineStr">
+        <is>
+          <t>503-5134375-2874203</t>
+        </is>
+      </c>
+      <c r="N20" s="27" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I21" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 18,259</t>
-        </is>
-      </c>
-      <c r="M21" s="32" t="inlineStr">
-        <is>
-          <t>17 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="I22" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 19,932</t>
+        </is>
+      </c>
+      <c r="M22" s="32" t="inlineStr">
+        <is>
+          <t>18 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="23"/>
     <row r="24"/>
     <row r="25"/>
@@ -2466,9 +2517,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="I21:L21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="I22:L22"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2581,29 +2632,29 @@
       </c>
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>KineShineX塑料除黄剂</t>
+          <t>KineShineX玻璃修复膏</t>
         </is>
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>100ml+毛巾</t>
+          <t>50g+海绵</t>
         </is>
       </c>
       <c r="D4" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="F4" s="33" t="n">
-        <v>46244.33587962963</v>
+        <v>46230.48587962963</v>
       </c>
       <c r="G4" s="33" t="n">
-        <v>46242</v>
+        <v>46232</v>
       </c>
       <c r="H4" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (2个)</t>
+          <t>库存充足 (1个)</t>
         </is>
       </c>
     </row>
@@ -2613,25 +2664,25 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>KineShineX玻璃修复膏</t>
+          <t>KineShineX塑料除黄剂</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>50g+海绵</t>
+          <t>100ml+毛巾</t>
         </is>
       </c>
       <c r="D5" s="28" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>46230.48587962963</v>
+        <v>46244.33587962963</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="H5" s="27" t="inlineStr">
         <is>
@@ -2711,7 +2762,7 @@
         </is>
       </c>
       <c r="D9" s="32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
@@ -3568,21 +3619,54 @@
         <v>1673</v>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="30" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="C20" s="36" t="inlineStr">
+        <is>
+          <t>503-5134375-2874203</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H20" s="34" t="n">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G21" s="31" t="n">
-        <v>97.59</v>
-      </c>
-      <c r="H21" s="35" t="n">
-        <v>18259</v>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="G22" s="31" t="n">
+        <v>104.26</v>
+      </c>
+      <c r="H22" s="35" t="n">
+        <v>19932</v>
+      </c>
+    </row>
     <row r="23"/>
     <row r="24"/>
     <row r="25"/>
@@ -3765,7 +3849,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3803,6 +3887,8 @@
     <hyperlink ref="C18" location="'📤销售表'!A18" display="250-3154848-2935021"/>
     <hyperlink ref="B19" location="'📥进货表'!A9" display="3316792152573008960"/>
     <hyperlink ref="C19" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B20" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C20" location="'📤销售表'!A20" display="503-5134375-2874203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增2笔出货订单 250-1961123 & 503-2776046 切蒜器
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2317,26 +2317,128 @@
       </c>
       <c r="N20" s="27" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="30" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D21" s="33" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G21" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J21" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K21" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L21" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>250-1961123-9212663</t>
+        </is>
+      </c>
+      <c r="N21" s="27" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D22" s="33" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J22" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K22" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L22" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M22" s="25" t="inlineStr">
+        <is>
+          <t>503-2776046-0470254</t>
+        </is>
+      </c>
+      <c r="N22" s="27" t="n"/>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I22" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 19,932</t>
-        </is>
-      </c>
-      <c r="M22" s="32" t="inlineStr">
-        <is>
-          <t>18 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24"/>
+      <c r="I24" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 21,790</t>
+        </is>
+      </c>
+      <c r="M24" s="32" t="inlineStr">
+        <is>
+          <t>20 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="25"/>
     <row r="26"/>
     <row r="27"/>
@@ -2517,9 +2619,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="I22:L22"/>
-    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="I24:L24"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2609,7 +2711,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.46</v>
@@ -2618,11 +2720,11 @@
         <v>46236.88541666666</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46243</v>
+        <v>46246</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (4个)</t>
+          <t>库存充足 (2个)</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2864,7 @@
         </is>
       </c>
       <c r="D9" s="32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
@@ -3591,32 +3693,32 @@
       </c>
       <c r="B19" s="36" t="inlineStr">
         <is>
-          <t>3316792152573008960</t>
+          <t>3315760069697054152</t>
         </is>
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>249-8279106-7397442</t>
+          <t>250-1961123-9212663</t>
         </is>
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
-          <t>塑料除黄剂 黄ばみ除去剤</t>
+          <t>切蒜器带透明收纳容器</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>100ml</t>
+          <t>绿色</t>
         </is>
       </c>
       <c r="F19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="29" t="n">
-        <v>6.67</v>
+        <v>4.57</v>
       </c>
       <c r="H19" s="34" t="n">
-        <v>1673</v>
+        <v>929</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
@@ -3625,50 +3727,116 @@
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
+          <t>3315760069697054152</t>
+        </is>
+      </c>
+      <c r="C20" s="36" t="inlineStr">
+        <is>
+          <t>503-2776046-0470254</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H20" s="34" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="36" t="inlineStr">
+        <is>
           <t>3316792152573008960</t>
         </is>
       </c>
-      <c r="C20" s="36" t="inlineStr">
+      <c r="C21" s="36" t="inlineStr">
+        <is>
+          <t>249-8279106-7397442</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H21" s="34" t="n">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>503-5134375-2874203</t>
         </is>
       </c>
-      <c r="D20" s="27" t="inlineStr">
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>塑料除黄剂 黄ばみ除去剤</t>
         </is>
       </c>
-      <c r="E20" s="27" t="inlineStr">
+      <c r="E22" s="27" t="inlineStr">
         <is>
           <t>100ml</t>
         </is>
       </c>
-      <c r="F20" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="29" t="n">
+      <c r="F22" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="29" t="n">
         <v>6.67</v>
       </c>
-      <c r="H20" s="34" t="n">
+      <c r="H22" s="34" t="n">
         <v>1673</v>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="30" t="inlineStr">
+    <row r="23"/>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G22" s="31" t="n">
-        <v>104.26</v>
-      </c>
-      <c r="H22" s="35" t="n">
-        <v>19932</v>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24"/>
+      <c r="G24" s="31" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="H24" s="35" t="n">
+        <v>21790</v>
+      </c>
+    </row>
     <row r="25"/>
     <row r="26"/>
     <row r="27"/>
@@ -3849,7 +4017,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -3885,10 +4053,14 @@
     <hyperlink ref="C17" location="'📤销售表'!A17" display="250-6902845-9205438"/>
     <hyperlink ref="B18" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C18" location="'📤销售表'!A18" display="250-3154848-2935021"/>
-    <hyperlink ref="B19" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C19" location="'📤销售表'!A19" display="249-8279106-7397442"/>
-    <hyperlink ref="B20" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C20" location="'📤销售表'!A20" display="503-5134375-2874203"/>
+    <hyperlink ref="B19" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C19" location="'📤销售表'!A21" display="250-1961123-9212663"/>
+    <hyperlink ref="B20" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C20" location="'📤销售表'!A22" display="503-2776046-0470254"/>
+    <hyperlink ref="B21" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C21" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B22" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C22" location="'📤销售表'!A20" display="503-5134375-2874203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增进货331637642022008960(10个) & 关联销售250-5218699
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -1060,23 +1060,64 @@
       </c>
       <c r="J9" s="27" t="n"/>
     </row>
-    <row r="10"/>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>1688</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>多功能不锈钢按压式压蒜器</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>按压压蒜器1个 绿色</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="29" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>331637642022008960</t>
+        </is>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J10" s="27" t="inlineStr">
+        <is>
+          <t>补货10个</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G11" s="31" t="n">
-        <v>135.2</v>
-      </c>
-      <c r="H11" s="32" t="inlineStr">
-        <is>
-          <t>7 笔进货</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
+      <c r="G12" s="31" t="n">
+        <v>184</v>
+      </c>
+      <c r="H12" s="32" t="inlineStr">
+        <is>
+          <t>8 笔进货</t>
+        </is>
+      </c>
+    </row>
     <row r="13"/>
     <row r="14"/>
     <row r="15"/>
@@ -1269,9 +1310,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="H12:J12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2421,25 +2462,76 @@
       </c>
       <c r="N22" s="27" t="n"/>
     </row>
-    <row r="23"/>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D23" s="33" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G23" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="34" t="n">
+        <v>699</v>
+      </c>
+      <c r="J23" s="34" t="n">
+        <v>64</v>
+      </c>
+      <c r="K23" s="34" t="n">
+        <v>169</v>
+      </c>
+      <c r="L23" s="34" t="n">
+        <v>929</v>
+      </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>250-5218699-2591031</t>
+        </is>
+      </c>
+      <c r="N23" s="27" t="n"/>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I24" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 21,790</t>
-        </is>
-      </c>
-      <c r="M24" s="32" t="inlineStr">
-        <is>
-          <t>20 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
+      <c r="I25" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 22,719</t>
+        </is>
+      </c>
+      <c r="M25" s="32" t="inlineStr">
+        <is>
+          <t>21 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="26"/>
     <row r="27"/>
     <row r="28"/>
@@ -2619,9 +2711,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="I24:L24"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="I25:L25"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2644,7 +2736,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2702,29 +2794,27 @@
       </c>
       <c r="B3" s="27" t="inlineStr">
         <is>
-          <t>多功能不锈钢压蒜器</t>
+          <t>多功能不锈钢按压式压蒜器</t>
         </is>
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>按压式2个装 绿色</t>
+          <t>按压压蒜器1个 绿色</t>
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>4.46</v>
+        <v>4.88</v>
       </c>
       <c r="F3" s="33" t="n">
-        <v>46236.88541666666</v>
-      </c>
-      <c r="G3" s="33" t="n">
-        <v>46246</v>
-      </c>
+        <v>46247</v>
+      </c>
+      <c r="G3" s="25" t="n"/>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (2个)</t>
+          <t>库存充足 (10个)</t>
         </is>
       </c>
     </row>
@@ -2766,25 +2856,25 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>KineShineX塑料除黄剂</t>
+          <t>多功能不锈钢压蒜器</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>100ml+毛巾</t>
+          <t>按压式2个装 绿色</t>
         </is>
       </c>
       <c r="D5" s="28" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>6.67</v>
+        <v>4.46</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>46244.33587962963</v>
+        <v>46236.88541666666</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="H5" s="27" t="inlineStr">
         <is>
@@ -2798,29 +2888,29 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>创意世界杯足球大力神杯</t>
+          <t>KineShineX塑料除黄剂</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>500ml透明圆形足球杯(牛皮纸盒包装)</t>
+          <t>100ml+毛巾</t>
         </is>
       </c>
       <c r="D6" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>5.9</v>
+        <v>6.67</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>46215.5080787037</v>
+        <v>46244.33587962963</v>
       </c>
       <c r="G6" s="33" t="n">
-        <v>46214</v>
+        <v>46244</v>
       </c>
       <c r="H6" s="27" t="inlineStr">
         <is>
-          <t>已售罄</t>
+          <t>库存充足 (1个)</t>
         </is>
       </c>
     </row>
@@ -2830,49 +2920,80 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
+          <t>创意世界杯足球大力神杯</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
+          <t>500ml透明圆形足球杯(牛皮纸盒包装)</t>
         </is>
       </c>
       <c r="D7" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="29" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>46215.5080787037</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <v>46214</v>
+      </c>
+      <c r="H7" s="27" t="inlineStr">
+        <is>
+          <t>已售罄</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>创意大力神杯世界杯足球玻璃啤酒杯</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>500ML电镀圆球形大力神杯（牛皮纸盒包装）</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F8" s="33" t="n">
         <v>46221.59108796297</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G8" s="33" t="n">
         <v>46221</v>
       </c>
-      <c r="H7" s="27" t="inlineStr">
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>已售罄</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+    <row r="9"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>📊 库存合计</t>
         </is>
       </c>
-      <c r="D9" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="32" t="inlineStr">
-        <is>
-          <t>5 种商品</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+      <c r="D10" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" s="32" t="inlineStr">
+        <is>
+          <t>6 种商品</t>
+        </is>
+      </c>
+    </row>
     <row r="11"/>
     <row r="12"/>
     <row r="13"/>
@@ -3067,8 +3188,8 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:H10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3761,32 +3882,32 @@
       </c>
       <c r="B21" s="36" t="inlineStr">
         <is>
-          <t>3316792152573008960</t>
+          <t>3315760069697054152</t>
         </is>
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
-          <t>249-8279106-7397442</t>
+          <t>250-5218699-2591031</t>
         </is>
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>塑料除黄剂 黄ばみ除去剤</t>
+          <t>切蒜器带透明收纳容器</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>100ml</t>
+          <t>绿色</t>
         </is>
       </c>
       <c r="F21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="29" t="n">
-        <v>6.67</v>
+        <v>4.57</v>
       </c>
       <c r="H21" s="34" t="n">
-        <v>1673</v>
+        <v>929</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
@@ -3800,7 +3921,7 @@
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>503-5134375-2874203</t>
+          <t>249-8279106-7397442</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
@@ -3823,21 +3944,54 @@
         <v>1673</v>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>503-5134375-2874203</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H23" s="34" t="n">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G24" s="31" t="n">
-        <v>113.4</v>
-      </c>
-      <c r="H24" s="35" t="n">
-        <v>21790</v>
-      </c>
-    </row>
-    <row r="25"/>
+      <c r="G25" s="31" t="n">
+        <v>117.97</v>
+      </c>
+      <c r="H25" s="35" t="n">
+        <v>22719</v>
+      </c>
+    </row>
     <row r="26"/>
     <row r="27"/>
     <row r="28"/>
@@ -4017,7 +4171,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -4057,10 +4211,12 @@
     <hyperlink ref="C19" location="'📤销售表'!A21" display="250-1961123-9212663"/>
     <hyperlink ref="B20" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C20" location="'📤销售表'!A22" display="503-2776046-0470254"/>
-    <hyperlink ref="B21" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C21" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B21" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C21" location="'📤销售表'!A23" display="250-5218699-2591031"/>
     <hyperlink ref="B22" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C22" location="'📤销售表'!A20" display="503-5134375-2874203"/>
+    <hyperlink ref="C22" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B23" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C23" location="'📤销售表'!A20" display="503-5134375-2874203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 新增出货订单 250-8757664 切蒜器x2
</commit_message>
<xml_diff>
--- a/购买记录/归档表格/购买记录_2026.xlsx
+++ b/购买记录/归档表格/购买记录_2026.xlsx
@@ -2514,25 +2514,76 @@
       </c>
       <c r="N23" s="27" t="n"/>
     </row>
-    <row r="24"/>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>Amazon日本站</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>46248</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>切蒜器带透明收纳容器</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>绿色</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="inlineStr">
+        <is>
+          <t>ba0010</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" s="34" t="n">
+        <v>1397</v>
+      </c>
+      <c r="J24" s="34" t="n">
+        <v>127</v>
+      </c>
+      <c r="K24" s="34" t="n">
+        <v>338</v>
+      </c>
+      <c r="L24" s="34" t="n">
+        <v>1857</v>
+      </c>
+      <c r="M24" s="25" t="inlineStr">
+        <is>
+          <t>250-8757664-8770260</t>
+        </is>
+      </c>
+      <c r="N24" s="27" t="n"/>
+    </row>
+    <row r="25"/>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="I25" s="32" t="inlineStr">
-        <is>
-          <t>总销售额: JPY 22,719</t>
-        </is>
-      </c>
-      <c r="M25" s="32" t="inlineStr">
-        <is>
-          <t>21 笔销售</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
+      <c r="I26" s="32" t="inlineStr">
+        <is>
+          <t>总销售额: JPY 24,576</t>
+        </is>
+      </c>
+      <c r="M26" s="32" t="inlineStr">
+        <is>
+          <t>22 笔销售</t>
+        </is>
+      </c>
+    </row>
     <row r="27"/>
     <row r="28"/>
     <row r="29"/>
@@ -2711,9 +2762,9 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="I25:L25"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="I26:L26"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2736,7 +2787,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2803,7 +2854,7 @@
         </is>
       </c>
       <c r="D3" s="28" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" s="29" t="n">
         <v>4.62</v>
@@ -2812,11 +2863,11 @@
         <v>46247</v>
       </c>
       <c r="G3" s="33" t="n">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>库存充足 (11个)</t>
+          <t>库存充足 (9个)</t>
         </is>
       </c>
     </row>
@@ -2956,7 +3007,7 @@
         </is>
       </c>
       <c r="D9" s="32" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
@@ -3887,32 +3938,32 @@
       </c>
       <c r="B22" s="36" t="inlineStr">
         <is>
-          <t>3316792152573008960</t>
+          <t>3315760069697054152</t>
         </is>
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>249-8279106-7397442</t>
+          <t>250-8757664-8770260</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>塑料除黄剂 黄ばみ除去剤</t>
+          <t>切蒜器带透明收纳容器</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>100ml</t>
+          <t>绿色</t>
         </is>
       </c>
       <c r="F22" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="29" t="n">
-        <v>6.67</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="H22" s="34" t="n">
-        <v>1673</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
@@ -3926,7 +3977,7 @@
       </c>
       <c r="C23" s="36" t="inlineStr">
         <is>
-          <t>503-5134375-2874203</t>
+          <t>249-8279106-7397442</t>
         </is>
       </c>
       <c r="D23" s="27" t="inlineStr">
@@ -3949,21 +4000,54 @@
         <v>1673</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>3316792152573008960</t>
+        </is>
+      </c>
+      <c r="C24" s="36" t="inlineStr">
+        <is>
+          <t>503-5134375-2874203</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>塑料除黄剂 黄ばみ除去剤</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H24" s="34" t="n">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>📊 合计</t>
         </is>
       </c>
-      <c r="G25" s="31" t="n">
-        <v>117.97</v>
-      </c>
-      <c r="H25" s="35" t="n">
-        <v>22719</v>
-      </c>
-    </row>
-    <row r="26"/>
+      <c r="G26" s="31" t="n">
+        <v>127.11</v>
+      </c>
+      <c r="H26" s="35" t="n">
+        <v>24576</v>
+      </c>
+    </row>
     <row r="27"/>
     <row r="28"/>
     <row r="29"/>
@@ -4142,7 +4226,7 @@
     <row r="202"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
@@ -4184,10 +4268,12 @@
     <hyperlink ref="C20" location="'📤销售表'!A22" display="503-2776046-0470254"/>
     <hyperlink ref="B21" location="'📥进货表'!A8" display="3315760069697054152"/>
     <hyperlink ref="C21" location="'📤销售表'!A23" display="250-5218699-2591031"/>
-    <hyperlink ref="B22" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C22" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B22" location="'📥进货表'!A8" display="3315760069697054152"/>
+    <hyperlink ref="C22" location="'📤销售表'!A24" display="250-8757664-8770260"/>
     <hyperlink ref="B23" location="'📥进货表'!A9" display="3316792152573008960"/>
-    <hyperlink ref="C23" location="'📤销售表'!A20" display="503-5134375-2874203"/>
+    <hyperlink ref="C23" location="'📤销售表'!A19" display="249-8279106-7397442"/>
+    <hyperlink ref="B24" location="'📥进货表'!A9" display="3316792152573008960"/>
+    <hyperlink ref="C24" location="'📤销售表'!A20" display="503-5134375-2874203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>